<commit_message>
Added appropriate swahili word for Yes in solar charger question (#136)
</commit_message>
<xml_diff>
--- a/forms/app/peer_mentor_checklist.xlsx
+++ b/forms/app/peer_mentor_checklist.xlsx
@@ -18,12 +18,12 @@
     <t>form_title</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
     <t>list_name</t>
   </si>
   <si>
-    <t>type</t>
-  </si>
-  <si>
     <t>form_id</t>
   </si>
   <si>
@@ -48,9 +48,57 @@
     <t>label::sw</t>
   </si>
   <si>
+    <t>required</t>
+  </si>
+  <si>
+    <t>relevant</t>
+  </si>
+  <si>
+    <t>appearance</t>
+  </si>
+  <si>
+    <t>read_only</t>
+  </si>
+  <si>
     <t>Peer Mentor Checklist</t>
   </si>
   <si>
+    <t>constraint</t>
+  </si>
+  <si>
+    <t>constraint_message::en</t>
+  </si>
+  <si>
+    <t>constraint_message::sw</t>
+  </si>
+  <si>
+    <t>calculation</t>
+  </si>
+  <si>
+    <t>choice_filter</t>
+  </si>
+  <si>
+    <t>hint::en</t>
+  </si>
+  <si>
+    <t>hint::sw</t>
+  </si>
+  <si>
+    <t>default</t>
+  </si>
+  <si>
+    <t>repeat_count</t>
+  </si>
+  <si>
+    <t>begin group</t>
+  </si>
+  <si>
+    <t>inputs</t>
+  </si>
+  <si>
+    <t>NO_LABEL</t>
+  </si>
+  <si>
     <t>peer_mentor_checklist</t>
   </si>
   <si>
@@ -96,63 +144,15 @@
     <t>chv_support_options</t>
   </si>
   <si>
-    <t>required</t>
-  </si>
-  <si>
-    <t>relevant</t>
-  </si>
-  <si>
-    <t>appearance</t>
-  </si>
-  <si>
-    <t>read_only</t>
-  </si>
-  <si>
-    <t>constraint</t>
-  </si>
-  <si>
-    <t>constraint_message::en</t>
-  </si>
-  <si>
-    <t>constraint_message::sw</t>
-  </si>
-  <si>
-    <t>calculation</t>
-  </si>
-  <si>
-    <t>choice_filter</t>
-  </si>
-  <si>
-    <t>hint::en</t>
-  </si>
-  <si>
-    <t>hint::sw</t>
-  </si>
-  <si>
-    <t>default</t>
-  </si>
-  <si>
     <t>tech_team</t>
   </si>
   <si>
-    <t>repeat_count</t>
-  </si>
-  <si>
     <t xml:space="preserve">Technology Team </t>
   </si>
   <si>
-    <t>begin group</t>
-  </si>
-  <si>
     <t xml:space="preserve">Timu ya Teknolojia </t>
   </si>
   <si>
-    <t>inputs</t>
-  </si>
-  <si>
-    <t>NO_LABEL</t>
-  </si>
-  <si>
     <t>chmt</t>
   </si>
   <si>
@@ -180,22 +180,22 @@
     <t>solar_charging</t>
   </si>
   <si>
+    <t>user</t>
+  </si>
+  <si>
     <t>no_solar_charger</t>
   </si>
   <si>
+    <t>string</t>
+  </si>
+  <si>
     <t>Does not have/need solar charger</t>
   </si>
   <si>
+    <t>contact_id</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hahitaji chaji ya sola </t>
-  </si>
-  <si>
-    <t>user</t>
-  </si>
-  <si>
-    <t>string</t>
-  </si>
-  <si>
-    <t>contact_id</t>
   </si>
   <si>
     <t>Contact ID of the logged in user</t>
@@ -702,6 +702,10 @@
       <name val="Arial"/>
     </font>
     <font>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="12.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -710,10 +714,6 @@
       <sz val="11.0"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
     </font>
     <font/>
     <font>
@@ -784,33 +784,33 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment vertical="bottom"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -829,7 +829,7 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -838,7 +838,7 @@
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -1109,7 +1109,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>8</v>
@@ -1117,62 +1117,62 @@
       <c r="C1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="9" t="s">
+      <c r="D1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="9" t="s">
-        <v>27</v>
-      </c>
-      <c r="F1" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="G1" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="I1" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>32</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="L1" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="N1" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>40</v>
+      <c r="E1" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="M1" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="N1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="O1" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="Q1" s="4" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2"/>
-      <c r="F2" s="12" t="b">
+      <c r="F2" s="11" t="b">
         <f>FALSE()</f>
         <v>0</v>
       </c>
@@ -1190,13 +1190,13 @@
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>45</v>
+        <v>27</v>
       </c>
       <c r="D3" s="2"/>
       <c r="E3" s="2"/>
@@ -1215,10 +1215,10 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>60</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>61</v>
@@ -1240,7 +1240,7 @@
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>62</v>
@@ -1265,7 +1265,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
@@ -1293,7 +1293,7 @@
         <v>65</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -1316,7 +1316,7 @@
         <v>65</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -1499,8 +1499,8 @@
       <c r="S14" s="18"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="s">
-        <v>42</v>
+      <c r="A15" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="B15" s="19" t="s">
         <v>83</v>
@@ -1513,7 +1513,7 @@
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
-      <c r="G15" s="9" t="s">
+      <c r="G15" s="4" t="s">
         <v>86</v>
       </c>
       <c r="H15" s="2"/>
@@ -1541,7 +1541,7 @@
         <v>90</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F16" s="21"/>
       <c r="G16" s="20"/>
@@ -1585,7 +1585,7 @@
         <v>96</v>
       </c>
       <c r="E17" s="20" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F17" s="21"/>
       <c r="G17" s="20"/>
@@ -1629,7 +1629,7 @@
         <v>101</v>
       </c>
       <c r="E18" s="20" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F18" s="21"/>
       <c r="G18" s="20"/>
@@ -1660,7 +1660,7 @@
       <c r="Z18" s="21"/>
     </row>
     <row r="19">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="4" t="s">
         <v>87</v>
       </c>
       <c r="B19" s="19" t="s">
@@ -1672,8 +1672,8 @@
       <c r="D19" s="19" t="s">
         <v>106</v>
       </c>
-      <c r="E19" s="9" t="s">
-        <v>16</v>
+      <c r="E19" s="4" t="s">
+        <v>32</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="23" t="s">
@@ -1740,7 +1740,7 @@
       </c>
       <c r="C21" s="19"/>
       <c r="D21" s="19"/>
-      <c r="E21" s="9"/>
+      <c r="E21" s="4"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
@@ -1763,8 +1763,8 @@
       <c r="B22" s="19" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="9"/>
-      <c r="E22" s="9"/>
+      <c r="C22" s="4"/>
+      <c r="E22" s="4"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
@@ -1780,7 +1780,7 @@
     </row>
     <row r="23">
       <c r="A23" s="19" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B23" s="19" t="s">
         <v>119</v>
@@ -1791,7 +1791,7 @@
       <c r="D23" s="19" t="s">
         <v>121</v>
       </c>
-      <c r="E23" s="9"/>
+      <c r="E23" s="4"/>
       <c r="F23" s="2"/>
       <c r="G23" s="27" t="s">
         <v>86</v>
@@ -1821,7 +1821,7 @@
         <v>125</v>
       </c>
       <c r="E24" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1850,15 +1850,15 @@
         <v>128</v>
       </c>
       <c r="E25" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F25" s="27" t="s">
         <v>129</v>
       </c>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
-      <c r="I25" s="9"/>
-      <c r="J25" s="9"/>
+      <c r="I25" s="4"/>
+      <c r="J25" s="4"/>
       <c r="K25" s="2"/>
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
@@ -1881,13 +1881,13 @@
         <v>132</v>
       </c>
       <c r="E26" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
-      <c r="I26" s="9"/>
-      <c r="J26" s="9"/>
+      <c r="I26" s="4"/>
+      <c r="J26" s="4"/>
       <c r="K26" s="2"/>
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
@@ -1910,15 +1910,15 @@
         <v>128</v>
       </c>
       <c r="E27" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F27" s="27" t="s">
         <v>134</v>
       </c>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
-      <c r="I27" s="9"/>
-      <c r="J27" s="9"/>
+      <c r="I27" s="4"/>
+      <c r="J27" s="4"/>
       <c r="K27" s="2"/>
       <c r="L27" s="2"/>
       <c r="M27" s="2"/>
@@ -1941,13 +1941,13 @@
         <v>137</v>
       </c>
       <c r="E28" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
-      <c r="I28" s="9"/>
-      <c r="J28" s="9"/>
+      <c r="I28" s="4"/>
+      <c r="J28" s="4"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
@@ -1970,15 +1970,15 @@
         <v>128</v>
       </c>
       <c r="E29" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F29" s="27" t="s">
         <v>139</v>
       </c>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
-      <c r="I29" s="9"/>
-      <c r="J29" s="9"/>
+      <c r="I29" s="4"/>
+      <c r="J29" s="4"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2001,7 +2001,7 @@
         <v>142</v>
       </c>
       <c r="E30" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -2030,15 +2030,15 @@
         <v>128</v>
       </c>
       <c r="E31" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F31" s="27" t="s">
         <v>144</v>
       </c>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
-      <c r="I31" s="9"/>
-      <c r="J31" s="9"/>
+      <c r="I31" s="4"/>
+      <c r="J31" s="4"/>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
       <c r="M31" s="2"/>
@@ -2061,7 +2061,7 @@
         <v>147</v>
       </c>
       <c r="E32" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -2090,15 +2090,15 @@
         <v>128</v>
       </c>
       <c r="E33" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F33" s="27" t="s">
         <v>149</v>
       </c>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
-      <c r="I33" s="9"/>
-      <c r="J33" s="9"/>
+      <c r="I33" s="4"/>
+      <c r="J33" s="4"/>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
       <c r="M33" s="2"/>
@@ -2121,7 +2121,7 @@
         <v>152</v>
       </c>
       <c r="E34" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
@@ -2150,15 +2150,15 @@
         <v>128</v>
       </c>
       <c r="E35" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F35" s="27" t="s">
         <v>154</v>
       </c>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
-      <c r="I35" s="9"/>
-      <c r="J35" s="9"/>
+      <c r="I35" s="4"/>
+      <c r="J35" s="4"/>
       <c r="K35" s="2"/>
       <c r="L35" s="2"/>
       <c r="M35" s="2"/>
@@ -2174,8 +2174,8 @@
       <c r="B36" s="19" t="s">
         <v>119</v>
       </c>
-      <c r="C36" s="9"/>
-      <c r="E36" s="9"/>
+      <c r="C36" s="4"/>
+      <c r="E36" s="4"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
@@ -2191,7 +2191,7 @@
     </row>
     <row r="37">
       <c r="A37" s="19" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B37" s="19" t="s">
         <v>155</v>
@@ -2231,7 +2231,7 @@
         <v>160</v>
       </c>
       <c r="E38" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -2260,15 +2260,15 @@
         <v>128</v>
       </c>
       <c r="E39" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F39" s="27" t="s">
         <v>162</v>
       </c>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
-      <c r="I39" s="9"/>
-      <c r="J39" s="9"/>
+      <c r="I39" s="4"/>
+      <c r="J39" s="4"/>
       <c r="K39" s="2"/>
       <c r="L39" s="2"/>
       <c r="M39" s="2"/>
@@ -2291,7 +2291,7 @@
         <v>165</v>
       </c>
       <c r="E40" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -2320,15 +2320,15 @@
         <v>128</v>
       </c>
       <c r="E41" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F41" s="27" t="s">
         <v>167</v>
       </c>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
-      <c r="I41" s="9"/>
-      <c r="J41" s="9"/>
+      <c r="I41" s="4"/>
+      <c r="J41" s="4"/>
       <c r="K41" s="2"/>
       <c r="L41" s="2"/>
       <c r="M41" s="2"/>
@@ -2351,7 +2351,7 @@
         <v>170</v>
       </c>
       <c r="E42" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
@@ -2380,15 +2380,15 @@
         <v>128</v>
       </c>
       <c r="E43" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F43" s="27" t="s">
         <v>172</v>
       </c>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
-      <c r="I43" s="9"/>
-      <c r="J43" s="9"/>
+      <c r="I43" s="4"/>
+      <c r="J43" s="4"/>
       <c r="K43" s="2"/>
       <c r="L43" s="2"/>
       <c r="M43" s="2"/>
@@ -2398,27 +2398,27 @@
       <c r="Q43" s="2"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="s">
+      <c r="A44" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B44" s="8" t="s">
+      <c r="B44" s="9" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B45" s="8" t="s">
+      <c r="A45" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>173</v>
       </c>
       <c r="C45" s="33" t="s">
         <v>174</v>
       </c>
-      <c r="D45" s="8" t="s">
+      <c r="D45" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="G45" s="8" t="s">
+      <c r="G45" s="9" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
         <v>178</v>
       </c>
       <c r="E46" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
@@ -2465,15 +2465,15 @@
         <v>128</v>
       </c>
       <c r="E47" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F47" s="27" t="s">
         <v>180</v>
       </c>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
-      <c r="I47" s="9"/>
-      <c r="J47" s="9"/>
+      <c r="I47" s="4"/>
+      <c r="J47" s="4"/>
       <c r="K47" s="2"/>
       <c r="L47" s="2"/>
       <c r="M47" s="2"/>
@@ -2496,7 +2496,7 @@
         <v>183</v>
       </c>
       <c r="E48" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
@@ -2525,15 +2525,15 @@
         <v>128</v>
       </c>
       <c r="E49" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F49" s="27" t="s">
         <v>185</v>
       </c>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
-      <c r="I49" s="9"/>
-      <c r="J49" s="9"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
       <c r="K49" s="2"/>
       <c r="L49" s="2"/>
       <c r="M49" s="2"/>
@@ -2556,7 +2556,7 @@
         <v>188</v>
       </c>
       <c r="E50" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
@@ -2585,15 +2585,15 @@
         <v>128</v>
       </c>
       <c r="E51" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F51" s="27" t="s">
         <v>190</v>
       </c>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
-      <c r="I51" s="9"/>
-      <c r="J51" s="9"/>
+      <c r="I51" s="4"/>
+      <c r="J51" s="4"/>
       <c r="K51" s="2"/>
       <c r="L51" s="2"/>
       <c r="M51" s="2"/>
@@ -2616,7 +2616,7 @@
         <v>193</v>
       </c>
       <c r="E52" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
@@ -2645,15 +2645,15 @@
         <v>128</v>
       </c>
       <c r="E53" s="19" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F53" s="27" t="s">
         <v>195</v>
       </c>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
-      <c r="I53" s="9"/>
-      <c r="J53" s="9"/>
+      <c r="I53" s="4"/>
+      <c r="J53" s="4"/>
       <c r="K53" s="2"/>
       <c r="L53" s="2"/>
       <c r="M53" s="2"/>
@@ -2663,47 +2663,47 @@
       <c r="Q53" s="2"/>
     </row>
     <row r="54">
-      <c r="A54" s="8" t="s">
+      <c r="A54" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B54" s="8" t="s">
+      <c r="B54" s="9" t="s">
         <v>173</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="8" t="s">
+      <c r="A55" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="B55" s="9" t="s">
+        <v>196</v>
+      </c>
+      <c r="C55" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D55" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="G55" s="9" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="B56" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="B55" s="8" t="s">
-        <v>196</v>
-      </c>
-      <c r="C55" s="8" t="s">
-        <v>197</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>198</v>
-      </c>
-      <c r="G55" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="8" t="s">
-        <v>199</v>
-      </c>
-      <c r="B56" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="C56" s="8" t="s">
+      <c r="C56" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="D56" s="8" t="s">
+      <c r="D56" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="E56" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F56" s="8"/>
+      <c r="E56" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="F56" s="9"/>
       <c r="I56" s="29" t="s">
         <v>202</v>
       </c>
@@ -2715,70 +2715,70 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="8" t="s">
+      <c r="A57" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B57" s="8" t="s">
+      <c r="B57" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="C57" s="8" t="s">
+      <c r="C57" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="D57" s="8" t="s">
+      <c r="D57" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="E57" s="8" t="s">
-        <v>16</v>
+      <c r="E57" s="9" t="s">
+        <v>32</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="8" t="s">
+      <c r="A58" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B58" s="8" t="s">
+      <c r="B58" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="C58" s="8" t="s">
+      <c r="C58" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="D58" s="8" t="s">
+      <c r="D58" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="E58" s="8" t="s">
-        <v>16</v>
+      <c r="E58" s="9" t="s">
+        <v>32</v>
       </c>
       <c r="F58" s="10" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="8" t="s">
+      <c r="A59" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="B59" s="8" t="s">
+      <c r="B59" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="C59" s="8" t="s">
+      <c r="C59" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="D59" s="8" t="s">
+      <c r="D59" s="9" t="s">
         <v>215</v>
       </c>
-      <c r="E59" s="8" t="s">
-        <v>16</v>
+      <c r="E59" s="9" t="s">
+        <v>32</v>
       </c>
       <c r="F59" s="10" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="8" t="s">
+      <c r="A60" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="B60" s="8" t="s">
+      <c r="B60" s="9" t="s">
         <v>196</v>
       </c>
     </row>
@@ -2802,199 +2802,199 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="s">
-        <v>1</v>
-      </c>
-      <c r="B1" s="6" t="s">
+      <c r="A1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="7" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="8" t="s">
-        <v>18</v>
+      <c r="A2" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>21</v>
+      <c r="A3" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D4" s="8" t="s">
-        <v>24</v>
+      <c r="A4" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>18</v>
+      <c r="A5" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="s">
-        <v>25</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="8" t="s">
-        <v>24</v>
+      <c r="A6" s="9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>41</v>
-      </c>
-      <c r="D7" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>43</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C8" s="8" t="s">
+      <c r="C8" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="D8" s="8" t="s">
+      <c r="D8" s="9" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B9" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B9" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="C9" s="8" t="s">
+      <c r="C9" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="D9" s="8" t="s">
+      <c r="D9" s="9" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="s">
+      <c r="A11" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B11" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="8" t="s">
-        <v>17</v>
+      <c r="B11" s="9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>34</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>21</v>
+      <c r="B12" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B13" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>24</v>
+      <c r="B13" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="s">
+      <c r="A14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="B14" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C14" s="11" t="s">
+      <c r="B14" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="D14" s="8" t="s">
-        <v>57</v>
+      <c r="C14" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -3054,17 +3054,17 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="7" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="7" t="s">
+      <c r="A2" s="6" t="s">
         <v>15</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2" s="8" t="s">
+        <v>31</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>

</xml_diff>

<commit_message>
Changed type of phone to tel
</commit_message>
<xml_diff>
--- a/forms/app/peer_mentor_checklist.xlsx
+++ b/forms/app/peer_mentor_checklist.xlsx
@@ -1,19 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\D-tree\config-dtree-newrepo\config-dtree\forms\app\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="4425" windowHeight="2115"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="survey" sheetId="1" r:id="rId4"/>
-    <sheet state="visible" name="choices" sheetId="2" r:id="rId5"/>
-    <sheet state="visible" name="settings" sheetId="3" r:id="rId6"/>
+    <sheet name="survey" sheetId="1" r:id="rId1"/>
+    <sheet name="choices" sheetId="2" r:id="rId2"/>
+    <sheet name="settings" sheetId="3" r:id="rId3"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="222">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="222">
   <si>
     <t>type</t>
   </si>
@@ -250,9 +258,6 @@
     <t>numbers</t>
   </si>
   <si>
-    <t>regex(.,'^0[0-9]{9}$')</t>
-  </si>
-  <si>
     <t>Use the following format 0XXXXXXXXX</t>
   </si>
   <si>
@@ -695,59 +700,71 @@
   </si>
   <si>
     <t>data</t>
+  </si>
+  <si>
+    <t>tel</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="12">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF1D1C1D"/>
       <name val="Slack-Lato"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Sans"/>
     </font>
     <font>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Roboto"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12.0"/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
-    <font/>
     <font>
-      <sz val="12.0"/>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Cambria"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
@@ -757,7 +774,7 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -773,147 +790,97 @@
     </fill>
   </fills>
   <borders count="3">
-    <border/>
     <border>
+      <left/>
       <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="38">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="top"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" readingOrder="0"/>
-    </xf>
-    <xf borderId="2" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1103,26 +1070,29 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z61"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="24.0"/>
-    <col customWidth="1" min="2" max="2" width="27.43"/>
-    <col customWidth="1" min="3" max="3" width="57.0"/>
-    <col customWidth="1" min="4" max="4" width="34.43"/>
-    <col customWidth="1" min="5" max="5" width="22.29"/>
-    <col customWidth="1" min="9" max="9" width="36.14"/>
-    <col customWidth="1" min="10" max="10" width="29.43"/>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="27.40625" customWidth="1"/>
+    <col min="3" max="3" width="57" customWidth="1"/>
+    <col min="4" max="4" width="34.40625" customWidth="1"/>
+    <col min="5" max="5" width="22.26953125" customWidth="1"/>
+    <col min="9" max="9" width="36.1328125" customWidth="1"/>
+    <col min="10" max="10" width="29.40625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" ht="13">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1175,7 +1145,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="13">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -1203,7 +1173,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3">
+    <row r="3" spans="1:26" ht="13">
       <c r="A3" s="1" t="s">
         <v>17</v>
       </c>
@@ -1228,7 +1198,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:26" ht="13">
       <c r="A4" s="1" t="s">
         <v>21</v>
       </c>
@@ -1253,7 +1223,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:26" ht="13">
       <c r="A5" s="1" t="s">
         <v>21</v>
       </c>
@@ -1278,7 +1248,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6">
+    <row r="6" spans="1:26" ht="13">
       <c r="A6" s="1" t="s">
         <v>21</v>
       </c>
@@ -1303,7 +1273,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7">
+    <row r="7" spans="1:26" ht="13">
       <c r="A7" s="1" t="s">
         <v>27</v>
       </c>
@@ -1326,7 +1296,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="1"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:26" ht="13">
       <c r="A8" s="1" t="s">
         <v>27</v>
       </c>
@@ -1349,7 +1319,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:26" ht="13">
       <c r="A9" s="1" t="s">
         <v>28</v>
       </c>
@@ -1376,7 +1346,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:26" ht="13">
       <c r="A10" s="1" t="s">
         <v>28</v>
       </c>
@@ -1403,7 +1373,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:26" ht="13">
       <c r="A11" s="1" t="s">
         <v>28</v>
       </c>
@@ -1430,7 +1400,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:26" ht="13">
       <c r="A12" s="2" t="s">
         <v>36</v>
       </c>
@@ -1462,7 +1432,7 @@
       <c r="Y12" s="10"/>
       <c r="Z12" s="10"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:26" ht="13">
       <c r="A13" s="2" t="s">
         <v>37</v>
       </c>
@@ -1494,7 +1464,7 @@
       <c r="Y13" s="10"/>
       <c r="Z13" s="10"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:26" ht="13">
       <c r="A14" s="8" t="s">
         <v>38</v>
       </c>
@@ -1523,7 +1493,7 @@
       <c r="R14" s="10"/>
       <c r="S14" s="10"/>
     </row>
-    <row r="15" ht="12.75" customHeight="1">
+    <row r="15" spans="1:26" ht="12.75" customHeight="1">
       <c r="A15" s="8" t="s">
         <v>42</v>
       </c>
@@ -1552,7 +1522,7 @@
       <c r="R15" s="10"/>
       <c r="S15" s="10"/>
     </row>
-    <row r="16">
+    <row r="16" spans="1:26" ht="13">
       <c r="A16" s="8" t="s">
         <v>46</v>
       </c>
@@ -1577,7 +1547,7 @@
       <c r="R16" s="10"/>
       <c r="S16" s="10"/>
     </row>
-    <row r="17">
+    <row r="17" spans="1:26" ht="13">
       <c r="A17" s="2" t="s">
         <v>17</v>
       </c>
@@ -1606,7 +1576,7 @@
       <c r="P17" s="1"/>
       <c r="Q17" s="1"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:26" ht="13">
       <c r="A18" s="13" t="s">
         <v>51</v>
       </c>
@@ -1650,7 +1620,7 @@
       <c r="Y18" s="14"/>
       <c r="Z18" s="14"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:26" ht="13">
       <c r="A19" s="13" t="s">
         <v>51</v>
       </c>
@@ -1694,7 +1664,7 @@
       <c r="Y19" s="14"/>
       <c r="Z19" s="14"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:26" ht="13">
       <c r="A20" s="13" t="s">
         <v>51</v>
       </c>
@@ -1738,9 +1708,9 @@
       <c r="Y20" s="14"/>
       <c r="Z20" s="14"/>
     </row>
-    <row r="21">
-      <c r="A21" s="2" t="s">
-        <v>51</v>
+    <row r="21" spans="1:26" ht="13">
+      <c r="A21" s="15" t="s">
+        <v>221</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>69</v>
@@ -1759,14 +1729,14 @@
         <v>72</v>
       </c>
       <c r="H21" s="1"/>
-      <c r="I21" s="15" t="s">
+      <c r="I21" s="15" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" s="15" t="s">
         <v>73</v>
       </c>
-      <c r="J21" s="15" t="s">
+      <c r="K21" s="15" t="s">
         <v>74</v>
-      </c>
-      <c r="K21" s="15" t="s">
-        <v>75</v>
       </c>
       <c r="L21" s="1"/>
       <c r="M21" s="1"/>
@@ -1775,21 +1745,21 @@
       <c r="P21" s="1"/>
       <c r="Q21" s="1"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:26" ht="13">
       <c r="A22" s="12" t="s">
         <v>51</v>
       </c>
       <c r="B22" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C22" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="D22" s="12" t="s">
         <v>77</v>
       </c>
-      <c r="D22" s="12" t="s">
+      <c r="E22" s="12" t="s">
         <v>78</v>
-      </c>
-      <c r="E22" s="12" t="s">
-        <v>79</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
@@ -1798,10 +1768,10 @@
         <v>56</v>
       </c>
       <c r="J22" s="16" t="s">
+        <v>79</v>
+      </c>
+      <c r="K22" s="17" t="s">
         <v>80</v>
-      </c>
-      <c r="K22" s="17" t="s">
-        <v>81</v>
       </c>
       <c r="L22" s="18"/>
       <c r="M22" s="1"/>
@@ -1810,14 +1780,15 @@
       <c r="P22" s="1"/>
       <c r="Q22" s="1"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:26" ht="13">
       <c r="A23" s="12" t="s">
         <v>27</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="2"/>
+      <c r="C23" s="35"/>
+      <c r="D23" s="36"/>
       <c r="E23" s="2"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
@@ -1832,18 +1803,18 @@
       <c r="P23" s="1"/>
       <c r="Q23" s="1"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:26" ht="13">
       <c r="A24" s="12" t="s">
         <v>17</v>
       </c>
       <c r="B24" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="C24" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="C24" s="12" t="s">
+      <c r="D24" s="12" t="s">
         <v>83</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>84</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="1"/>
@@ -1861,18 +1832,18 @@
       <c r="P24" s="1"/>
       <c r="Q24" s="1"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:26" ht="14.25">
       <c r="A25" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B25" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="12" t="s">
+      <c r="C25" s="21" t="s">
         <v>86</v>
       </c>
-      <c r="C25" s="21" t="s">
+      <c r="D25" s="22" t="s">
         <v>87</v>
-      </c>
-      <c r="D25" s="22" t="s">
-        <v>88</v>
       </c>
       <c r="E25" s="12" t="s">
         <v>55</v>
@@ -1890,24 +1861,24 @@
       <c r="P25" s="1"/>
       <c r="Q25" s="1"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:26" ht="14.25">
       <c r="A26" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B26" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="C26" s="22" t="s">
         <v>89</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="D26" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="D26" s="22" t="s">
+      <c r="E26" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F26" s="19" t="s">
         <v>91</v>
-      </c>
-      <c r="E26" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F26" s="19" t="s">
-        <v>92</v>
       </c>
       <c r="G26" s="1"/>
       <c r="H26" s="1"/>
@@ -1921,18 +1892,18 @@
       <c r="P26" s="1"/>
       <c r="Q26" s="1"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:26" ht="14.25">
       <c r="A27" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B27" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C27" s="22" t="s">
         <v>93</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="D27" s="22" t="s">
         <v>94</v>
-      </c>
-      <c r="D27" s="22" t="s">
-        <v>95</v>
       </c>
       <c r="E27" s="12" t="s">
         <v>55</v>
@@ -1950,24 +1921,24 @@
       <c r="P27" s="1"/>
       <c r="Q27" s="1"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:26" ht="14.25">
       <c r="A28" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B28" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="C28" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D28" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F28" s="19" t="s">
         <v>96</v>
-      </c>
-      <c r="C28" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D28" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E28" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F28" s="19" t="s">
-        <v>97</v>
       </c>
       <c r="G28" s="1"/>
       <c r="H28" s="1"/>
@@ -1981,18 +1952,18 @@
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:26" ht="14.25">
       <c r="A29" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B29" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="C29" s="22" t="s">
         <v>98</v>
       </c>
-      <c r="C29" s="22" t="s">
+      <c r="D29" s="21" t="s">
         <v>99</v>
-      </c>
-      <c r="D29" s="21" t="s">
-        <v>100</v>
       </c>
       <c r="E29" s="12" t="s">
         <v>55</v>
@@ -2010,24 +1981,24 @@
       <c r="P29" s="1"/>
       <c r="Q29" s="1"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:26" ht="14.25">
       <c r="A30" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B30" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D30" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F30" s="19" t="s">
         <v>101</v>
-      </c>
-      <c r="C30" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D30" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E30" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F30" s="19" t="s">
-        <v>102</v>
       </c>
       <c r="G30" s="1"/>
       <c r="H30" s="1"/>
@@ -2041,18 +2012,18 @@
       <c r="P30" s="1"/>
       <c r="Q30" s="1"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:26" ht="14.25">
       <c r="A31" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B31" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C31" s="22" t="s">
+      <c r="D31" s="22" t="s">
         <v>104</v>
-      </c>
-      <c r="D31" s="22" t="s">
-        <v>105</v>
       </c>
       <c r="E31" s="12" t="s">
         <v>55</v>
@@ -2070,24 +2041,24 @@
       <c r="P31" s="1"/>
       <c r="Q31" s="1"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:26" ht="14.25">
       <c r="A32" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B32" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="C32" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D32" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F32" s="19" t="s">
         <v>106</v>
-      </c>
-      <c r="C32" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D32" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E32" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F32" s="19" t="s">
-        <v>107</v>
       </c>
       <c r="G32" s="1"/>
       <c r="H32" s="1"/>
@@ -2101,18 +2072,18 @@
       <c r="P32" s="1"/>
       <c r="Q32" s="1"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:17" ht="13">
       <c r="A33" s="23" t="s">
+        <v>107</v>
+      </c>
+      <c r="B33" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="C33" s="21" t="s">
         <v>109</v>
       </c>
-      <c r="C33" s="21" t="s">
+      <c r="D33" s="21" t="s">
         <v>110</v>
-      </c>
-      <c r="D33" s="21" t="s">
-        <v>111</v>
       </c>
       <c r="E33" s="12" t="s">
         <v>55</v>
@@ -2130,24 +2101,24 @@
       <c r="P33" s="1"/>
       <c r="Q33" s="1"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:17" ht="14.25">
       <c r="A34" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B34" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="C34" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D34" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E34" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F34" s="19" t="s">
         <v>112</v>
-      </c>
-      <c r="C34" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D34" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F34" s="19" t="s">
-        <v>113</v>
       </c>
       <c r="G34" s="1"/>
       <c r="H34" s="1"/>
@@ -2161,18 +2132,18 @@
       <c r="P34" s="1"/>
       <c r="Q34" s="1"/>
     </row>
-    <row r="35">
+    <row r="35" spans="1:17" ht="14.25">
       <c r="A35" s="23" t="s">
+        <v>113</v>
+      </c>
+      <c r="B35" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="B35" s="12" t="s">
+      <c r="C35" s="21" t="s">
         <v>115</v>
       </c>
-      <c r="C35" s="21" t="s">
+      <c r="D35" s="22" t="s">
         <v>116</v>
-      </c>
-      <c r="D35" s="22" t="s">
-        <v>117</v>
       </c>
       <c r="E35" s="12" t="s">
         <v>55</v>
@@ -2190,24 +2161,24 @@
       <c r="P35" s="1"/>
       <c r="Q35" s="1"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:17" ht="14.25">
       <c r="A36" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B36" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="C36" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D36" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E36" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F36" s="19" t="s">
         <v>118</v>
-      </c>
-      <c r="C36" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D36" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E36" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F36" s="19" t="s">
-        <v>119</v>
       </c>
       <c r="G36" s="1"/>
       <c r="H36" s="1"/>
@@ -2221,14 +2192,15 @@
       <c r="P36" s="1"/>
       <c r="Q36" s="1"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:17" ht="13">
       <c r="A37" s="12" t="s">
         <v>27</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C37" s="2"/>
+        <v>81</v>
+      </c>
+      <c r="C37" s="35"/>
+      <c r="D37" s="36"/>
       <c r="E37" s="2"/>
       <c r="F37" s="1"/>
       <c r="G37" s="1"/>
@@ -2243,18 +2215,18 @@
       <c r="P37" s="1"/>
       <c r="Q37" s="1"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:17" ht="13">
       <c r="A38" s="12" t="s">
         <v>17</v>
       </c>
       <c r="B38" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="C38" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="D38" s="12" t="s">
         <v>121</v>
-      </c>
-      <c r="D38" s="12" t="s">
-        <v>122</v>
       </c>
       <c r="F38" s="1"/>
       <c r="G38" s="12" t="s">
@@ -2271,18 +2243,18 @@
       <c r="P38" s="1"/>
       <c r="Q38" s="1"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:17" ht="14.25">
       <c r="A39" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B39" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="C39" s="22" t="s">
         <v>123</v>
       </c>
-      <c r="C39" s="22" t="s">
+      <c r="D39" s="22" t="s">
         <v>124</v>
-      </c>
-      <c r="D39" s="22" t="s">
-        <v>125</v>
       </c>
       <c r="E39" s="12" t="s">
         <v>55</v>
@@ -2300,24 +2272,24 @@
       <c r="P39" s="1"/>
       <c r="Q39" s="1"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:17" ht="14.25">
       <c r="A40" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B40" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="C40" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D40" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E40" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F40" s="19" t="s">
         <v>126</v>
-      </c>
-      <c r="C40" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D40" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E40" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F40" s="19" t="s">
-        <v>127</v>
       </c>
       <c r="G40" s="1"/>
       <c r="H40" s="1"/>
@@ -2331,18 +2303,18 @@
       <c r="P40" s="1"/>
       <c r="Q40" s="1"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:17" ht="14.25">
       <c r="A41" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B41" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="C41" s="22" t="s">
         <v>128</v>
       </c>
-      <c r="C41" s="22" t="s">
+      <c r="D41" s="22" t="s">
         <v>129</v>
-      </c>
-      <c r="D41" s="22" t="s">
-        <v>130</v>
       </c>
       <c r="E41" s="12" t="s">
         <v>55</v>
@@ -2360,24 +2332,24 @@
       <c r="P41" s="1"/>
       <c r="Q41" s="1"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:17" ht="14.25">
       <c r="A42" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B42" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="C42" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D42" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F42" s="19" t="s">
         <v>131</v>
-      </c>
-      <c r="C42" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D42" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E42" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F42" s="19" t="s">
-        <v>132</v>
       </c>
       <c r="G42" s="1"/>
       <c r="H42" s="1"/>
@@ -2391,18 +2363,18 @@
       <c r="P42" s="1"/>
       <c r="Q42" s="1"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:17" ht="14.25">
       <c r="A43" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B43" s="12" t="s">
+        <v>132</v>
+      </c>
+      <c r="C43" s="22" t="s">
         <v>133</v>
       </c>
-      <c r="C43" s="22" t="s">
+      <c r="D43" s="21" t="s">
         <v>134</v>
-      </c>
-      <c r="D43" s="21" t="s">
-        <v>135</v>
       </c>
       <c r="E43" s="12" t="s">
         <v>55</v>
@@ -2420,24 +2392,24 @@
       <c r="P43" s="1"/>
       <c r="Q43" s="1"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:17" ht="14.25">
       <c r="A44" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B44" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="C44" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D44" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F44" s="19" t="s">
         <v>136</v>
-      </c>
-      <c r="C44" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D44" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E44" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F44" s="19" t="s">
-        <v>137</v>
       </c>
       <c r="G44" s="1"/>
       <c r="H44" s="1"/>
@@ -2451,43 +2423,43 @@
       <c r="P44" s="1"/>
       <c r="Q44" s="1"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:17" ht="13">
       <c r="A45" s="24" t="s">
         <v>27</v>
       </c>
       <c r="B45" s="24" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="46">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" ht="13">
       <c r="A46" s="24" t="s">
         <v>17</v>
       </c>
       <c r="B46" s="24" t="s">
+        <v>137</v>
+      </c>
+      <c r="C46" s="25" t="s">
         <v>138</v>
       </c>
-      <c r="C46" s="25" t="s">
+      <c r="D46" s="24" t="s">
         <v>139</v>
-      </c>
-      <c r="D46" s="24" t="s">
-        <v>140</v>
       </c>
       <c r="G46" s="24" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="47">
+    <row r="47" spans="1:17" ht="14.25">
       <c r="A47" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B47" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C47" s="21" t="s">
         <v>141</v>
       </c>
-      <c r="C47" s="21" t="s">
+      <c r="D47" s="22" t="s">
         <v>142</v>
-      </c>
-      <c r="D47" s="22" t="s">
-        <v>143</v>
       </c>
       <c r="E47" s="12" t="s">
         <v>55</v>
@@ -2505,24 +2477,24 @@
       <c r="P47" s="1"/>
       <c r="Q47" s="1"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:17" ht="14.25">
       <c r="A48" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B48" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="C48" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D48" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E48" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F48" s="19" t="s">
         <v>144</v>
-      </c>
-      <c r="C48" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D48" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E48" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F48" s="19" t="s">
-        <v>145</v>
       </c>
       <c r="G48" s="1"/>
       <c r="H48" s="1"/>
@@ -2536,18 +2508,18 @@
       <c r="P48" s="1"/>
       <c r="Q48" s="1"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:17" ht="13">
       <c r="A49" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B49" s="12" t="s">
+        <v>145</v>
+      </c>
+      <c r="C49" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="C49" s="21" t="s">
+      <c r="D49" s="21" t="s">
         <v>147</v>
-      </c>
-      <c r="D49" s="21" t="s">
-        <v>148</v>
       </c>
       <c r="E49" s="12" t="s">
         <v>55</v>
@@ -2565,24 +2537,24 @@
       <c r="P49" s="1"/>
       <c r="Q49" s="1"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:17" ht="14.25">
       <c r="A50" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B50" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="C50" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D50" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E50" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F50" s="19" t="s">
         <v>149</v>
-      </c>
-      <c r="C50" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D50" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E50" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F50" s="19" t="s">
-        <v>150</v>
       </c>
       <c r="G50" s="1"/>
       <c r="H50" s="1"/>
@@ -2596,18 +2568,18 @@
       <c r="P50" s="1"/>
       <c r="Q50" s="1"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:17" ht="13">
       <c r="A51" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B51" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C51" s="21" t="s">
         <v>151</v>
       </c>
-      <c r="C51" s="21" t="s">
+      <c r="D51" s="21" t="s">
         <v>152</v>
-      </c>
-      <c r="D51" s="21" t="s">
-        <v>153</v>
       </c>
       <c r="E51" s="12" t="s">
         <v>55</v>
@@ -2625,24 +2597,24 @@
       <c r="P51" s="1"/>
       <c r="Q51" s="1"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:17" ht="14.25">
       <c r="A52" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B52" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="C52" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D52" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E52" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F52" s="19" t="s">
         <v>154</v>
-      </c>
-      <c r="C52" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D52" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E52" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F52" s="19" t="s">
-        <v>155</v>
       </c>
       <c r="G52" s="1"/>
       <c r="H52" s="1"/>
@@ -2656,18 +2628,18 @@
       <c r="P52" s="1"/>
       <c r="Q52" s="1"/>
     </row>
-    <row r="53">
+    <row r="53" spans="1:17" ht="14.25">
       <c r="A53" s="20" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B53" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="C53" s="22" t="s">
         <v>156</v>
       </c>
-      <c r="C53" s="22" t="s">
+      <c r="D53" s="21" t="s">
         <v>157</v>
-      </c>
-      <c r="D53" s="21" t="s">
-        <v>158</v>
       </c>
       <c r="E53" s="12" t="s">
         <v>55</v>
@@ -2685,24 +2657,24 @@
       <c r="P53" s="1"/>
       <c r="Q53" s="1"/>
     </row>
-    <row r="54">
+    <row r="54" spans="1:17" ht="14.25">
       <c r="A54" s="20" t="s">
         <v>51</v>
       </c>
       <c r="B54" s="12" t="s">
+        <v>158</v>
+      </c>
+      <c r="C54" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="D54" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="E54" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F54" s="19" t="s">
         <v>159</v>
-      </c>
-      <c r="C54" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="D54" s="22" t="s">
-        <v>91</v>
-      </c>
-      <c r="E54" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="F54" s="19" t="s">
-        <v>160</v>
       </c>
       <c r="G54" s="1"/>
       <c r="H54" s="1"/>
@@ -2716,124 +2688,124 @@
       <c r="P54" s="1"/>
       <c r="Q54" s="1"/>
     </row>
-    <row r="55">
+    <row r="55" spans="1:17" ht="13">
       <c r="A55" s="24" t="s">
         <v>27</v>
       </c>
       <c r="B55" s="24" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="56">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="56" spans="1:17" ht="13">
       <c r="A56" s="24" t="s">
         <v>17</v>
       </c>
       <c r="B56" s="24" t="s">
+        <v>160</v>
+      </c>
+      <c r="C56" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="C56" s="24" t="s">
+      <c r="D56" s="24" t="s">
         <v>162</v>
-      </c>
-      <c r="D56" s="24" t="s">
-        <v>163</v>
       </c>
       <c r="G56" s="24" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="57">
+    <row r="57" spans="1:17" ht="13">
       <c r="A57" s="24" t="s">
+        <v>163</v>
+      </c>
+      <c r="B57" s="24" t="s">
         <v>164</v>
       </c>
-      <c r="B57" s="24" t="s">
+      <c r="C57" s="24" t="s">
         <v>165</v>
       </c>
-      <c r="C57" s="24" t="s">
+      <c r="D57" s="24" t="s">
         <v>166</v>
-      </c>
-      <c r="D57" s="24" t="s">
-        <v>167</v>
       </c>
       <c r="E57" s="24" t="s">
         <v>55</v>
       </c>
       <c r="F57" s="24"/>
       <c r="I57" s="20" t="s">
+        <v>167</v>
+      </c>
+      <c r="J57" s="20" t="s">
         <v>168</v>
       </c>
-      <c r="J57" s="20" t="s">
+      <c r="K57" s="26" t="s">
         <v>169</v>
       </c>
-      <c r="K57" s="26" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="58">
+    </row>
+    <row r="58" spans="1:17" ht="13">
       <c r="A58" s="24" t="s">
         <v>51</v>
       </c>
       <c r="B58" s="24" t="s">
+        <v>170</v>
+      </c>
+      <c r="C58" s="24" t="s">
         <v>171</v>
       </c>
-      <c r="C58" s="24" t="s">
+      <c r="D58" s="24" t="s">
         <v>172</v>
       </c>
-      <c r="D58" s="24" t="s">
+      <c r="E58" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="F58" s="27" t="s">
         <v>173</v>
       </c>
-      <c r="E58" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="F58" s="27" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="59">
+    </row>
+    <row r="59" spans="1:17" ht="13">
       <c r="A59" s="24" t="s">
         <v>51</v>
       </c>
       <c r="B59" s="24" t="s">
+        <v>174</v>
+      </c>
+      <c r="C59" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="C59" s="24" t="s">
+      <c r="D59" s="24" t="s">
         <v>176</v>
       </c>
-      <c r="D59" s="24" t="s">
+      <c r="E59" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="F59" s="27" t="s">
         <v>177</v>
       </c>
-      <c r="E59" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="F59" s="27" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="60">
+    </row>
+    <row r="60" spans="1:17" ht="13">
       <c r="A60" s="24" t="s">
         <v>51</v>
       </c>
       <c r="B60" s="24" t="s">
+        <v>178</v>
+      </c>
+      <c r="C60" s="24" t="s">
         <v>179</v>
       </c>
-      <c r="C60" s="24" t="s">
+      <c r="D60" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="D60" s="24" t="s">
+      <c r="E60" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="F60" s="27" t="s">
         <v>181</v>
       </c>
-      <c r="E60" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="F60" s="27" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="61">
+    </row>
+    <row r="61" spans="1:17" ht="13">
       <c r="A61" s="24" t="s">
         <v>27</v>
       </c>
       <c r="B61" s="24" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2841,23 +2813,24 @@
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C37:D37"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:D18"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="18.29"/>
+    <col min="1" max="1" width="18.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:4">
       <c r="A1" s="28" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B1" s="29" t="s">
         <v>1</v>
@@ -2869,278 +2842,279 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:4" ht="15.75" customHeight="1">
       <c r="A2" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C2" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="B2" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="24" t="s">
+      <c r="D2" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="D2" s="24" t="s">
+    </row>
+    <row r="3" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A3" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="B3" s="24" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="24" t="s">
+      <c r="C3" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" s="24" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A4" s="24" t="s">
+        <v>183</v>
+      </c>
+      <c r="B4" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="D4" s="24" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" customHeight="1">
+      <c r="A5" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="B5" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="D5" s="24" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="13">
+      <c r="A6" s="24" t="s">
+        <v>192</v>
+      </c>
+      <c r="B6" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="C6" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="13">
+      <c r="A7" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B7" s="24" t="s">
+        <v>193</v>
+      </c>
+      <c r="C7" s="24" t="s">
+        <v>194</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="13">
+      <c r="A8" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B8" s="24" t="s">
+        <v>196</v>
+      </c>
+      <c r="C8" s="24" t="s">
+        <v>197</v>
+      </c>
+      <c r="D8" s="24" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="13">
+      <c r="A9" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B9" s="24" t="s">
+        <v>199</v>
+      </c>
+      <c r="C9" s="24" t="s">
+        <v>200</v>
+      </c>
+      <c r="D9" s="24" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="13">
+      <c r="A10" s="27" t="s">
+        <v>164</v>
+      </c>
+      <c r="B10" s="24" t="s">
+        <v>201</v>
+      </c>
+      <c r="C10" s="24" t="s">
+        <v>202</v>
+      </c>
+      <c r="D10" s="24" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="13">
+      <c r="A11" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="D11" s="30" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="13">
+      <c r="A12" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>186</v>
+      </c>
+      <c r="C12" s="30" t="s">
         <v>187</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="D12" s="30" t="s">
         <v>188</v>
       </c>
-      <c r="D3" s="24" t="s">
+    </row>
+    <row r="13" spans="1:4" ht="13">
+      <c r="A13" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B13" s="24" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="24" t="s">
+      <c r="C13" s="24" t="s">
+        <v>190</v>
+      </c>
+      <c r="D13" s="30" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="13">
+      <c r="A14" s="24" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>204</v>
+      </c>
+      <c r="C14" s="30" t="s">
+        <v>205</v>
+      </c>
+      <c r="D14" s="24" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="13">
+      <c r="A15" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B15" s="24" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="B4" s="24" t="s">
+      <c r="D15" s="24" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="13">
+      <c r="A16" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B16" s="24" t="s">
+        <v>186</v>
+      </c>
+      <c r="C16" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="D16" s="24" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="13">
+      <c r="A17" s="24" t="s">
+        <v>207</v>
+      </c>
+      <c r="B17" s="24" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="24" t="s">
         <v>190</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="D17" s="24" t="s">
         <v>191</v>
       </c>
-      <c r="D4" s="24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="24" t="s">
-        <v>193</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>185</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="s">
-        <v>193</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>194</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>195</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>197</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>198</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>200</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>201</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="27" t="s">
-        <v>165</v>
-      </c>
-      <c r="B10" s="24" t="s">
-        <v>202</v>
-      </c>
-      <c r="C10" s="24" t="s">
-        <v>203</v>
-      </c>
-      <c r="D10" s="24" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>185</v>
-      </c>
-      <c r="D11" s="30" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B12" s="30" t="s">
-        <v>187</v>
-      </c>
-      <c r="C12" s="30" t="s">
-        <v>188</v>
-      </c>
-      <c r="D12" s="30" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B13" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="D13" s="30" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="24" t="s">
-        <v>115</v>
-      </c>
-      <c r="B14" s="24" t="s">
-        <v>205</v>
-      </c>
-      <c r="C14" s="30" t="s">
-        <v>206</v>
-      </c>
-      <c r="D14" s="24" t="s">
+    </row>
+    <row r="18" spans="1:4" ht="13">
+      <c r="A18" s="24" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="24" t="s">
+      <c r="B18" s="30" t="s">
         <v>208</v>
       </c>
-      <c r="B15" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>185</v>
-      </c>
-      <c r="D15" s="24" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B16" s="24" t="s">
-        <v>187</v>
-      </c>
-      <c r="C16" s="24" t="s">
-        <v>188</v>
-      </c>
-      <c r="D16" s="24" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B17" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>191</v>
-      </c>
-      <c r="D17" s="24" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="B18" s="30" t="s">
+      <c r="C18" s="30" t="s">
         <v>209</v>
       </c>
-      <c r="C18" s="30" t="s">
+      <c r="D18" s="30" t="s">
         <v>210</v>
       </c>
-      <c r="D18" s="30" t="s">
-        <v>211</v>
-      </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <dimension ref="A1:Z2"/>
+  <sheetFormatPr defaultColWidth="14.40625" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="19.43"/>
-    <col customWidth="1" min="2" max="2" width="20.29"/>
+    <col min="1" max="1" width="19.40625" customWidth="1"/>
+    <col min="2" max="2" width="20.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:26" ht="15.75" customHeight="1">
       <c r="A1" s="31" t="s">
+        <v>211</v>
+      </c>
+      <c r="B1" s="31" t="s">
         <v>212</v>
       </c>
-      <c r="B1" s="31" t="s">
+      <c r="C1" s="31" t="s">
         <v>213</v>
       </c>
-      <c r="C1" s="31" t="s">
+      <c r="D1" s="31" t="s">
         <v>214</v>
       </c>
-      <c r="D1" s="31" t="s">
+      <c r="E1" s="31" t="s">
         <v>215</v>
       </c>
-      <c r="E1" s="31" t="s">
+      <c r="F1" s="32" t="s">
         <v>216</v>
-      </c>
-      <c r="F1" s="32" t="s">
-        <v>217</v>
       </c>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -3163,18 +3137,19 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2">
+    <row r="2" spans="1:26" ht="15.75" customHeight="1">
       <c r="A2" s="33" t="s">
+        <v>217</v>
+      </c>
+      <c r="B2" s="37" t="s">
         <v>218</v>
       </c>
-      <c r="B2" s="33" t="s">
+      <c r="C2" s="36"/>
+      <c r="D2" s="34" t="s">
         <v>219</v>
       </c>
-      <c r="D2" s="34" t="s">
+      <c r="E2" s="34" t="s">
         <v>220</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>221</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
@@ -3202,6 +3177,6 @@
   <mergeCells count="1">
     <mergeCell ref="B2:C2"/>
   </mergeCells>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>